<commit_message>
Audit data sources and add repair tooling
</commit_message>
<xml_diff>
--- a/data/correct_datas.xlsx
+++ b/data/correct_datas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>11010000</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -458,7 +458,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1006</t>
+          <t>10060000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -475,12 +475,250 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1701</t>
+          <t>17010000</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fruit Juice Mixed</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>22029990</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Orange Juice 200ML</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20099000</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Harpic Toilet Cleaner 500ML</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>34022090</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Harpic Power Plus</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>34022090</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fruit Jam</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>20079990</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mixed Fruit Jam</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>20079990</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cashew Cookie</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>19053100</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Horlicks Womens</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>21069099</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>VKC Chappal</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>64029990</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Basmati Rice</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10063020</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sesame Oil</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15155091</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gingelly Oil</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15155091</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Colgate Toothpaste</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>33061020</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Shampoo</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>33051090</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>

</xml_diff>